<commit_message>
Updates to Mexico power sector: 1) Updated start year capacity, mandated additions, and retirements to align with the first modeled year being 2021 and the first non-calibrated year being 2024; 2) Updated power sources used in least cost dispatch to inclue fuel oil plants; 3) Updated MCF values to correctly cover downtime, not average capacity factors, Updated RAF for capacity to include wind and solad; 4) Updated share of costs that must be covered to be deemed profitable to to 1 for all values.
</commit_message>
<xml_diff>
--- a/InputData/elec/ESUfRaLCD/Elec Sources Used for Rlbty and Lst Cst Dsptch.xlsx
+++ b/InputData/elec/ESUfRaLCD/Elec Sources Used for Rlbty and Lst Cst Dsptch.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28318"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rod\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\Mexico\Models\eps-mexico\InputData\elec\ESUfRaLCD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="8_{86AAAC9A-42F8-4F88-8DC2-3D590C5E19A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1C720BE2-4D80-4AED-BF64-A4C4805F0218}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F46B243B-45B0-48F3-953D-C4CC9BD06AFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="2" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
+    <workbookView xWindow="25230" yWindow="2385" windowWidth="24510" windowHeight="17910" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="50">
   <si>
     <t>ESUFRaLCD Electricity Sources Used for Reliability and Least Cost Dispatch</t>
   </si>
@@ -185,13 +185,16 @@
   </si>
   <si>
     <t>municipal solid waste</t>
+  </si>
+  <si>
+    <t>heavy or residual fuel oil</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -249,9 +252,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -289,7 +292,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -395,7 +398,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -537,7 +540,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -546,14 +549,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A1D3264-BEAA-43D0-A5CC-06C5D3B72BE0}">
   <dimension ref="A1:B30"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -561,7 +564,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -569,112 +572,112 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:1">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:1">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="19" spans="1:1">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:1">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:1">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="22" spans="1:1">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:1">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="24" spans="1:1">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:1">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="26" spans="1:1">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="27" spans="1:1">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:1">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:1">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>26</v>
       </c>
@@ -690,7 +693,7 @@
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
   <dimension ref="A1:I82"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
@@ -699,7 +702,7 @@
     <col min="9" max="9" width="24.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -713,7 +716,7 @@
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>30</v>
       </c>
@@ -726,7 +729,7 @@
         <v>natural gas combined cycle power plants</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -739,7 +742,7 @@
         <v>onshore wind power plants</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>32</v>
       </c>
@@ -752,7 +755,7 @@
         <v>solar PV power plants</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>33</v>
       </c>
@@ -765,7 +768,7 @@
         <v>petroleum power plants</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -778,7 +781,7 @@
         <v>natural gas peaker power plants</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -790,7 +793,7 @@
         <v>hard coal w ccs power plants</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -802,7 +805,7 @@
         <v>natural gas combined cycle w ccs power plants</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -814,7 +817,7 @@
         <v>lignite w ccs power plants</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>40</v>
       </c>
@@ -827,7 +830,7 @@
         <v>hydrogen combustion turbine power plants</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>41</v>
       </c>
@@ -840,7 +843,7 @@
         <v>hydrogen combined cycle power plants</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -850,7 +853,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -860,7 +863,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -870,7 +873,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -880,7 +883,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -890,7 +893,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="2:3">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -900,7 +903,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="2:3">
+    <row r="18" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -910,7 +913,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="2:3">
+    <row r="19" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B19" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -920,7 +923,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="2:3">
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B20" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -930,7 +933,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="2:3">
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -940,7 +943,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="2:3">
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -950,7 +953,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="2:3">
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -960,355 +963,355 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="2:3">
+    <row r="24" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C24" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="25" spans="2:3">
+    <row r="25" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C25" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="26" spans="2:3">
+    <row r="26" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C26" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="27" spans="2:3">
+    <row r="27" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="28" spans="2:3">
+    <row r="28" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C28" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="29" spans="2:3">
+    <row r="29" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C29" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="30" spans="2:3">
+    <row r="30" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="31" spans="2:3">
+    <row r="31" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C31" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="32" spans="2:3">
+    <row r="32" spans="2:3" x14ac:dyDescent="0.25">
       <c r="C32" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="33" spans="3:3">
+    <row r="33" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C33" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="34" spans="3:3">
+    <row r="34" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C34" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="35" spans="3:3">
+    <row r="35" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C35" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="36" spans="3:3">
+    <row r="36" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C36" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="37" spans="3:3">
+    <row r="37" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C37" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="38" spans="3:3">
+    <row r="38" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C38" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="39" spans="3:3">
+    <row r="39" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C39" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="40" spans="3:3">
+    <row r="40" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C40" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="41" spans="3:3">
+    <row r="41" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C41" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="42" spans="3:3">
+    <row r="42" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C42" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="43" spans="3:3">
+    <row r="43" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C43" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="44" spans="3:3">
+    <row r="44" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C44" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="45" spans="3:3">
+    <row r="45" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C45" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="46" spans="3:3">
+    <row r="46" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C46" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="47" spans="3:3">
+    <row r="47" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C47" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="48" spans="3:3">
+    <row r="48" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C48" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="49" spans="3:3">
+    <row r="49" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C49" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="50" spans="3:3">
+    <row r="50" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C50" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="51" spans="3:3">
+    <row r="51" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C51" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="52" spans="3:3">
+    <row r="52" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C52" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="53" spans="3:3">
+    <row r="53" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C53" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="54" spans="3:3">
+    <row r="54" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C54" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="55" spans="3:3">
+    <row r="55" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C55" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="56" spans="3:3">
+    <row r="56" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C56" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="57" spans="3:3">
+    <row r="57" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C57" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="58" spans="3:3">
+    <row r="58" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C58" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="59" spans="3:3">
+    <row r="59" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C59" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="60" spans="3:3">
+    <row r="60" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C60" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="61" spans="3:3">
+    <row r="61" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C61" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="62" spans="3:3">
+    <row r="62" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C62" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="63" spans="3:3">
+    <row r="63" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C63" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="64" spans="3:3">
+    <row r="64" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C64" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="65" spans="3:3">
+    <row r="65" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C65" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="66" spans="3:3">
+    <row r="66" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C66" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="67" spans="3:3">
+    <row r="67" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C67" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="68" spans="3:3">
+    <row r="68" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C68" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="69" spans="3:3">
+    <row r="69" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C69" t="str">
         <f t="shared" ref="C69:C82" si="2">IF(A69="","",CONCATENATE(A69," power plants"))</f>
         <v/>
       </c>
     </row>
-    <row r="70" spans="3:3">
+    <row r="70" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C70" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="71" spans="3:3">
+    <row r="71" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C71" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="72" spans="3:3">
+    <row r="72" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C72" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="73" spans="3:3">
+    <row r="73" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C73" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="74" spans="3:3">
+    <row r="74" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C74" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="75" spans="3:3">
+    <row r="75" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C75" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="76" spans="3:3">
+    <row r="76" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C76" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="77" spans="3:3">
+    <row r="77" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C77" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="78" spans="3:3">
+    <row r="78" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C78" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="79" spans="3:3">
+    <row r="79" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C79" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="80" spans="3:3">
+    <row r="80" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C80" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="81" spans="3:3">
+    <row r="81" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C81" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
-    <row r="82" spans="3:3">
+    <row r="82" spans="3:3" x14ac:dyDescent="0.25">
       <c r="C82" t="str">
         <f t="shared" si="2"/>
         <v/>
@@ -1324,14 +1327,14 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <dimension ref="A1:C15"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>27</v>
       </c>
@@ -1342,7 +1345,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>43</v>
       </c>
@@ -1355,20 +1358,20 @@
         <v>hard coal dispatch</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>44</v>
       </c>
       <c r="B3" t="str">
-        <f t="shared" ref="B3:B14" si="0">IF(A3="","",CONCATENATE(A3," es"))</f>
+        <f t="shared" ref="B3:B15" si="0">IF(A3="","",CONCATENATE(A3," es"))</f>
         <v>natural gas steam turbine es</v>
       </c>
       <c r="C3" t="str">
-        <f t="shared" ref="C3:C14" si="1">IF(A3="","",CONCATENATE(A3," dispatch"))</f>
+        <f t="shared" ref="C3:C15" si="1">IF(A3="","",CONCATENATE(A3," dispatch"))</f>
         <v>natural gas steam turbine dispatch</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>30</v>
       </c>
@@ -1381,7 +1384,7 @@
         <v>natural gas combined cycle dispatch</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>45</v>
       </c>
@@ -1392,7 +1395,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>33</v>
       </c>
@@ -1405,7 +1408,7 @@
         <v>petroleum dispatch</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>34</v>
       </c>
@@ -1418,7 +1421,7 @@
         <v>natural gas peaker dispatch</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>47</v>
       </c>
@@ -1431,77 +1434,90 @@
         <v>lignite dispatch</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>heavy or residual fuel oil es</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="1"/>
+        <v>heavy or residual fuel oil dispatch</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>48</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>municipal solid waste es</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C10" t="str">
         <f t="shared" si="1"/>
         <v>municipal solid waste dispatch</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
-      <c r="A10" t="s">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>35</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B11" t="s">
         <v>36</v>
       </c>
-      <c r="C10" t="str">
+      <c r="C11" t="str">
         <f t="shared" si="1"/>
         <v>hard coal w ccs dispatch</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
-      <c r="A11" t="s">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>37</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B12" t="s">
         <v>38</v>
       </c>
-      <c r="C11" t="str">
+      <c r="C12" t="str">
         <f t="shared" si="1"/>
         <v>natural gas combined cycle w ccs dispatch</v>
       </c>
     </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>39</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B13" t="s">
         <v>22</v>
       </c>
-      <c r="C12" t="str">
+      <c r="C13" t="str">
         <f t="shared" si="1"/>
         <v>lignite w ccs dispatch</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
-      <c r="A13" t="s">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>40</v>
       </c>
-      <c r="B13" t="str">
+      <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>hydrogen combustion turbine es</v>
       </c>
-      <c r="C13" t="str">
+      <c r="C14" t="str">
         <f t="shared" si="1"/>
         <v>hydrogen combustion turbine dispatch</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
-      <c r="A14" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
         <v>41</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v>hydrogen combined cycle es</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C15" t="str">
         <f t="shared" si="1"/>
         <v>hydrogen combined cycle dispatch</v>
       </c>
@@ -1512,6 +1528,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009A9DAB439B36DB4795F39C4E722C7BC4" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="44674c89fa9bc5e97a878a6680c46188">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="79748b23-d81a-423e-9112-21109dc864e6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="447839a363ea5a12024b5bf1ab53ed90" ns2:_="">
     <xsd:import namespace="79748b23-d81a-423e-9112-21109dc864e6"/>
@@ -1655,29 +1686,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AFA3F65-15F1-45B6-85EF-A78DE3771DB4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2058A945-B0A7-420B-8284-DCA9A2E0F0D0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A32AF48B-7BAE-4EB5-A14C-3507F28D9AB0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A32AF48B-7BAE-4EB5-A14C-3507F28D9AB0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2058A945-B0A7-420B-8284-DCA9A2E0F0D0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2AFA3F65-15F1-45B6-85EF-A78DE3771DB4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="79748b23-d81a-423e-9112-21109dc864e6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>